<commit_message>
Updates from the vps
</commit_message>
<xml_diff>
--- a/ExcelToXMLConverter/resources/SIGIDOC_ENG_BG_2025.03.26.test.xlsx
+++ b/ExcelToXMLConverter/resources/SIGIDOC_ENG_BG_2025.03.26.test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/repos/codecrew/SigiDoc/ExcelToXMLConverter/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700D32B0-D9C9-A54E-A4D8-D03FFE768560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCD9A2C-7F05-AC4C-ABFE-66B6EC87E790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19820" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>

</xml_diff>